<commit_message>
feat: update flash card
</commit_message>
<xml_diff>
--- a/public/vocabulary_sample.xlsx
+++ b/public/vocabulary_sample.xlsx
@@ -3,8 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Vocabulary" sheetId="1" r:id="rId1"/>
-    <sheet name="Hướng dẫn" sheetId="2" r:id="rId2"/>
+    <sheet name="Từ vựng IELTS" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -398,15 +397,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:I4"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" customWidth="1"/>
-    <col min="5" max="5" width="50.83203125" customWidth="1"/>
-    <col min="6" max="6" width="30.83203125" customWidth="1"/>
-    <col min="7" max="7" width="30.83203125" customWidth="1"/>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="25.83203125" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="60.83203125" customWidth="1"/>
+    <col min="7" max="7" width="60.83203125" customWidth="1"/>
+    <col min="8" max="8" width="25.83203125" customWidth="1"/>
+    <col min="9" max="9" width="25.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -417,243 +418,117 @@
         <v>Vietnamese</v>
       </c>
       <c r="C1" t="str">
+        <v>Level</v>
+      </c>
+      <c r="D1" t="str">
         <v>Phiên âm</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Từ loại</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Example</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
+        <v>Nghĩa ví dụ</v>
+      </c>
+      <c r="H1" t="str">
         <v>Synonyms</v>
       </c>
-      <c r="G1" t="str">
+      <c r="I1" t="str">
         <v>Antonyms</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>abundant</v>
+        <v>ambiguous</v>
       </c>
       <c r="B2" t="str">
-        <v>dồi dào, phong phú</v>
+        <v>mơ hồ, không rõ ràng</v>
       </c>
       <c r="C2" t="str">
-        <v>/əˈbʌn.dənt/</v>
+        <v>C1</v>
       </c>
       <c r="D2" t="str">
+        <v>/æmˈbɪɡ.ju.əs/</v>
+      </c>
+      <c r="E2" t="str">
         <v>adjective</v>
       </c>
-      <c r="E2" t="str">
-        <v>There is an abundant supply of fresh water in this region.</v>
-      </c>
       <c r="F2" t="str">
-        <v>plentiful, ample, copious</v>
+        <v>The instructions were ambiguous and confusing.</v>
       </c>
       <c r="G2" t="str">
-        <v>scarce, rare, limited</v>
+        <v>Các hướng dẫn rất mơ hồ và khó hiểu.</v>
+      </c>
+      <c r="H2" t="str">
+        <v>unclear, vague</v>
+      </c>
+      <c r="I2" t="str">
+        <v>clear, obvious</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ambiguous</v>
+        <v>diligent</v>
       </c>
       <c r="B3" t="str">
-        <v>mơ hồ, không rõ ràng</v>
+        <v>siêng năng, cần mẫn</v>
       </c>
       <c r="C3" t="str">
-        <v>/æmˈbɪɡ.ju.əs/</v>
+        <v>B2</v>
       </c>
       <c r="D3" t="str">
+        <v>/ˈdɪl.ɪ.dʒənt/</v>
+      </c>
+      <c r="E3" t="str">
         <v>adjective</v>
       </c>
-      <c r="E3" t="str">
-        <v>The instructions were ambiguous and confusing.</v>
-      </c>
       <c r="F3" t="str">
-        <v>vague, unclear, obscure</v>
+        <v>He is a diligent student who always completes his homework.</v>
       </c>
       <c r="G3" t="str">
-        <v>clear, definite, explicit</v>
+        <v>Anh ấy là một học sinh siêng năng luôn hoàn thành bài tập về nhà.</v>
+      </c>
+      <c r="H3" t="str">
+        <v>hardworking, industrious</v>
+      </c>
+      <c r="I3" t="str">
+        <v>lazy</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>advocate</v>
+        <v>procrastinate</v>
       </c>
       <c r="B4" t="str">
-        <v>ủng hộ; người ủng hộ</v>
+        <v>trì hoãn</v>
       </c>
       <c r="C4" t="str">
-        <v>/ˈæd.və.keɪt/</v>
+        <v>C1</v>
       </c>
       <c r="D4" t="str">
-        <v>verb / noun</v>
+        <v>/prəˈkræs.tɪ.neɪt/</v>
       </c>
       <c r="E4" t="str">
-        <v>She advocates for better education policies.</v>
+        <v>verb</v>
       </c>
       <c r="F4" t="str">
-        <v>support, promote, champion</v>
+        <v>Don't procrastinate when you have an important deadline.</v>
       </c>
       <c r="G4" t="str">
-        <v>oppose, resist, reject</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>alleviate</v>
-      </c>
-      <c r="B5" t="str">
-        <v>giảm bớt, làm nhẹ đi</v>
-      </c>
-      <c r="C5" t="str">
-        <v>/əˈliː.vi.eɪt/</v>
-      </c>
-      <c r="D5" t="str">
-        <v>verb</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Medication can help alleviate the pain.</v>
-      </c>
-      <c r="F5" t="str">
-        <v>relieve, ease, reduce</v>
-      </c>
-      <c r="G5" t="str">
-        <v>aggravate, worsen, increase</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>coherent</v>
-      </c>
-      <c r="B6" t="str">
-        <v>mạch lạc, nhất quán</v>
-      </c>
-      <c r="C6" t="str">
-        <v>/kəʊˈhɪə.rənt/</v>
-      </c>
-      <c r="D6" t="str">
-        <v>adjective</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Please give a coherent explanation of your argument.</v>
-      </c>
-      <c r="F6" t="str">
-        <v>logical, consistent, clear</v>
-      </c>
-      <c r="G6" t="str">
-        <v>incoherent, illogical, confused</v>
+        <v>Đừng trì hoãn khi bạn có một hạn chót quan trọng.</v>
+      </c>
+      <c r="H4" t="str">
+        <v>delay, postpone</v>
+      </c>
+      <c r="I4" t="str">
+        <v>hasten, hurry</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
-  <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="45.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Cột</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Bắt buộc</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Mô tả</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>English</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Có ✅</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Từ tiếng Anh</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Vietnamese</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Có ✅</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Nghĩa tiếng Việt</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Phiên âm</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Không</v>
-      </c>
-      <c r="C4" t="str">
-        <v>IPA phonetics, ví dụ: /ˈwɜːd/</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Từ loại</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Không</v>
-      </c>
-      <c r="C5" t="str">
-        <v>noun, verb, adjective, adverb, phrase...</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Example</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Không</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Câu ví dụ sử dụng từ</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Synonyms</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Không</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Từ đồng nghĩa, cách nhau bằng dấu phẩy</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Antonyms</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Không</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Từ trái nghĩa, cách nhau bằng dấu phẩy</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add YoutubeExercise component with integrated vocabulary note-taking and Excel export functionality
</commit_message>
<xml_diff>
--- a/public/vocabulary_sample.xlsx
+++ b/public/vocabulary_sample.xlsx
@@ -1,55 +1,148 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Từ vựng IELTS" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Vocabulary" state="visible" r:id="rId4"/>
   </sheets>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="34">
+  <si>
+    <t>English</t>
+  </si>
+  <si>
+    <t>Vietnamese</t>
+  </si>
+  <si>
+    <t>Level</t>
+  </si>
+  <si>
+    <t>Phiên âm</t>
+  </si>
+  <si>
+    <t>Từ loại</t>
+  </si>
+  <si>
+    <t>Example</t>
+  </si>
+  <si>
+    <t>Nghĩa ví dụ</t>
+  </si>
+  <si>
+    <t>Synonyms</t>
+  </si>
+  <si>
+    <t>Antonyms</t>
+  </si>
+  <si>
+    <t>ambiguous</t>
+  </si>
+  <si>
+    <t>mơ hồ, không rõ ràng</t>
+  </si>
+  <si>
+    <t>C1</t>
+  </si>
+  <si>
+    <t>/æmˈbɪɡ.ju.əs/</t>
+  </si>
+  <si>
+    <t>adjective</t>
+  </si>
+  <si>
+    <t>The instructions were ambiguous and confusing.</t>
+  </si>
+  <si>
+    <t>Các hướng dẫn rất mơ hồ và khó hiểu.</t>
+  </si>
+  <si>
+    <t>unclear, vague</t>
+  </si>
+  <si>
+    <t>clear, obvious</t>
+  </si>
+  <si>
+    <t>diligent</t>
+  </si>
+  <si>
+    <t>siêng năng, cần mẫn</t>
+  </si>
+  <si>
+    <t>B2</t>
+  </si>
+  <si>
+    <t>/ˈdɪl.ɪ.dʒənt/</t>
+  </si>
+  <si>
+    <t>He is a diligent student who always completes his homework.</t>
+  </si>
+  <si>
+    <t>Anh ấy là một học sinh siêng năng luôn hoàn thành bài tập về nhà.</t>
+  </si>
+  <si>
+    <t>hardworking, industrious</t>
+  </si>
+  <si>
+    <t>lazy</t>
+  </si>
+  <si>
+    <t>procrastinate</t>
+  </si>
+  <si>
+    <t>trì hoãn</t>
+  </si>
+  <si>
+    <t>/prəˈkræs.tɪ.neɪt/</t>
+  </si>
+  <si>
+    <t>verb</t>
+  </si>
+  <si>
+    <t>Don't procrastinate when you have an important deadline.</t>
+  </si>
+  <si>
+    <t>Đừng trì hoãn khi bạn có một hạn chót quan trọng.</t>
+  </si>
+  <si>
+    <t>delay, postpone</t>
+  </si>
+  <si>
+    <t>hasten, hurry</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4F81BD"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -64,14 +157,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,139 +500,137 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I4"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="25.83203125" customWidth="1"/>
-    <col min="3" max="3" width="8.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="60.83203125" customWidth="1"/>
-    <col min="7" max="7" width="60.83203125" customWidth="1"/>
-    <col min="8" max="8" width="25.83203125" customWidth="1"/>
-    <col min="9" max="9" width="25.83203125" customWidth="1"/>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="7" width="40" customWidth="1"/>
+    <col min="8" max="9" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>English</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Vietnamese</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Level</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Phiên âm</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Từ loại</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Example</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Nghĩa ví dụ</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Synonyms</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Antonyms</v>
+    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>ambiguous</v>
-      </c>
-      <c r="B2" t="str">
-        <v>mơ hồ, không rõ ràng</v>
-      </c>
-      <c r="C2" t="str">
-        <v>C1</v>
-      </c>
-      <c r="D2" t="str">
-        <v>/æmˈbɪɡ.ju.əs/</v>
-      </c>
-      <c r="E2" t="str">
-        <v>adjective</v>
-      </c>
-      <c r="F2" t="str">
-        <v>The instructions were ambiguous and confusing.</v>
-      </c>
-      <c r="G2" t="str">
-        <v>Các hướng dẫn rất mơ hồ và khó hiểu.</v>
-      </c>
-      <c r="H2" t="str">
-        <v>unclear, vague</v>
-      </c>
-      <c r="I2" t="str">
-        <v>clear, obvious</v>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>diligent</v>
-      </c>
-      <c r="B3" t="str">
-        <v>siêng năng, cần mẫn</v>
-      </c>
-      <c r="C3" t="str">
-        <v>B2</v>
-      </c>
-      <c r="D3" t="str">
-        <v>/ˈdɪl.ɪ.dʒənt/</v>
-      </c>
-      <c r="E3" t="str">
-        <v>adjective</v>
-      </c>
-      <c r="F3" t="str">
-        <v>He is a diligent student who always completes his homework.</v>
-      </c>
-      <c r="G3" t="str">
-        <v>Anh ấy là một học sinh siêng năng luôn hoàn thành bài tập về nhà.</v>
-      </c>
-      <c r="H3" t="str">
-        <v>hardworking, industrious</v>
-      </c>
-      <c r="I3" t="str">
-        <v>lazy</v>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" t="s">
+        <v>25</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>procrastinate</v>
-      </c>
-      <c r="B4" t="str">
-        <v>trì hoãn</v>
-      </c>
-      <c r="C4" t="str">
-        <v>C1</v>
-      </c>
-      <c r="D4" t="str">
-        <v>/prəˈkræs.tɪ.neɪt/</v>
-      </c>
-      <c r="E4" t="str">
-        <v>verb</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Don't procrastinate when you have an important deadline.</v>
-      </c>
-      <c r="G4" t="str">
-        <v>Đừng trì hoãn khi bạn có một hạn chót quan trọng.</v>
-      </c>
-      <c r="H4" t="str">
-        <v>delay, postpone</v>
-      </c>
-      <c r="I4" t="str">
-        <v>hasten, hurry</v>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H4" t="s">
+        <v>32</v>
+      </c>
+      <c r="I4" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
-  </ignoredErrors>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>